<commit_message>
Substitution : alignement des mappings CDA sur les évolutions du modèle métier
- Dispensation : substitution.type et substitution.reason remplacent substitutionOccurred
- Prescription : substitution.allowed[x] cible le code de FRCDAAutorisationSubstitution 0390a704980aca97c878a658e1976cfeaae9a814
</commit_message>
<xml_diff>
--- a/majMapping/ig/FRMedicationDispenseLMCDAFHIR.xlsx
+++ b/majMapping/ig/FRMedicationDispenseLMCDAFHIR.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="127">
   <si>
     <t>Property</t>
   </si>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-08T12:48:01+00:00</t>
+    <t>2026-10-08T13:13:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -162,10 +162,13 @@
     <t>Supply.quantity</t>
   </si>
   <si>
-    <t>FRLMMedicationDispense.substitutionOccurred</t>
-  </si>
-  <si>
-    <t>Supply.entryRelationship:frActeSubstitution</t>
+    <t>FRLMMedicationDispense.substitution.type</t>
+  </si>
+  <si>
+    <t>source-is-broader-than-target</t>
+  </si>
+  <si>
+    <t>Supply.entryRelationship:frActeSubstitution.code</t>
   </si>
   <si>
     <t>FRCDAActeSubstitution</t>
@@ -231,7 +234,13 @@
     <t>MedicationDispense.whenHandedOver</t>
   </si>
   <si>
-    <t>MedicationDispense.substitution.wasSubstituted</t>
+    <t>MedicationDispense.substitution.type</t>
+  </si>
+  <si>
+    <t>FRLMMedicationDispense.substitution.reason[x]</t>
+  </si>
+  <si>
+    <t>MedicationDispense.substitution.reason</t>
   </si>
   <si>
     <t>MedicationDispense.dosageInstruction</t>
@@ -768,43 +777,43 @@
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E11" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -814,7 +823,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -845,7 +854,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -860,10 +869,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -875,20 +884,20 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -901,20 +910,20 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -927,7 +936,7 @@
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -940,7 +949,7 @@
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -953,20 +962,20 @@
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -979,35 +988,48 @@
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14" s="2"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>55</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E15" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -1038,7 +1060,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -1047,7 +1069,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -1055,228 +1077,228 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E19" s="2"/>
     </row>
@@ -1309,7 +1331,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -1318,7 +1340,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -1326,287 +1348,287 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D21" t="s" s="2">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" t="s" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D22" t="s" s="2">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E23" s="2"/>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D24" t="s" s="2">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E24" s="2"/>
     </row>

</xml_diff>